<commit_message>
Sync backlog Estado for H-01 and H-02 to Publicado
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UWjkDqFXp236QdbmxGtwXE
</commit_message>
<xml_diff>
--- a/content/blog/Backlog_Blog_Continental_Media.xlsx
+++ b/content/blog/Backlog_Blog_Continental_Media.xlsx
@@ -13260,203 +13260,203 @@
       </c>
     </row>
     <row r="102">
-      <c r="A102" t="inlineStr">
+      <c r="A102" s="27" t="inlineStr">
         <is>
           <t>H-01</t>
         </is>
       </c>
-      <c r="B102" t="inlineStr">
+      <c r="B102" s="27" t="inlineStr">
         <is>
           <t>Editorial</t>
         </is>
       </c>
-      <c r="C102" t="inlineStr">
+      <c r="C102" s="27" t="inlineStr">
         <is>
           <t>Historia de la publicidad en México</t>
         </is>
       </c>
-      <c r="D102" t="inlineStr">
+      <c r="D102" s="27" t="inlineStr">
         <is>
           <t>Estrategia de marketing y contenidos</t>
         </is>
       </c>
-      <c r="E102" t="inlineStr">
+      <c r="E102" s="27" t="inlineStr">
         <is>
           <t>historia de la publicidad en méxico</t>
         </is>
       </c>
-      <c r="F102" t="inlineStr">
+      <c r="F102" s="27" t="inlineStr">
         <is>
           <t>Informacional</t>
         </is>
       </c>
-      <c r="G102" t="inlineStr">
+      <c r="G102" s="27" t="inlineStr">
         <is>
           <t>TOFU</t>
         </is>
       </c>
-      <c r="H102" t="inlineStr">
+      <c r="H102" s="27" t="inlineStr">
         <is>
           <t>Conservar el posicionamiento ya ganado de la URL original (202 clics/16m) con una versión 2026 ampliada y verificada.</t>
         </is>
       </c>
-      <c r="I102" t="inlineStr">
+      <c r="I102" s="27" t="inlineStr">
         <is>
           <t>General</t>
         </is>
       </c>
-      <c r="J102" t="inlineStr">
+      <c r="J102" s="27" t="inlineStr">
         <is>
           <t>México</t>
         </is>
       </c>
-      <c r="K102" t="inlineStr">
+      <c r="K102" s="27" t="inlineStr">
         <is>
           <t>Actualizar v2026 (misma URL)</t>
         </is>
       </c>
-      <c r="L102" t="inlineStr">
+      <c r="L102" s="27" t="inlineStr">
         <is>
           <t>https://www.continentalmedia.com.mx/2013/04/historia-de-la-publicidad-en-mexico/</t>
         </is>
       </c>
-      <c r="N102" t="inlineStr">
+      <c r="N102" s="27" t="inlineStr">
         <is>
           <t>Migración SEO — ruta heredada, ver migracion/LEEME_transicion_seo.md §5</t>
         </is>
       </c>
-      <c r="P102" t="inlineStr">
+      <c r="P102" s="27" t="inlineStr">
         <is>
           <t>Estrategia de marketing 360</t>
         </is>
       </c>
-      <c r="R102" t="inlineStr">
+      <c r="R102" s="27" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="T102">
+      <c r="T102" s="27">
         <f>CHOOSE(MONTH(X102),"Ene","Feb","Mar","Abr","May","Jun","Jul","Ago","Sep","Oct","Nov","Dic")&amp;" "&amp;YEAR(X102)</f>
         <v/>
       </c>
-      <c r="W102" t="inlineStr">
-        <is>
-          <t>En revisión</t>
+      <c r="W102" s="27" t="inlineStr">
+        <is>
+          <t>Publicado</t>
         </is>
       </c>
       <c r="X102" s="49" t="n">
         <v>46322</v>
       </c>
-      <c r="Y102">
+      <c r="Y102" s="27">
         <f>CHOOSE(WEEKDAY(X102,2),"lunes","martes","miércoles","jueves","viernes","sábado","domingo")</f>
         <v/>
       </c>
-      <c r="Z102">
+      <c r="Z102" s="27">
         <f>INT((X102-MIN($X$2:$X$103))/7)+1</f>
         <v/>
       </c>
-      <c r="AA102">
+      <c r="AA102" s="27">
         <f>IF(X102=MIN($X$2:$X$103),"Lanzamiento","Calendario semanal")</f>
         <v/>
       </c>
     </row>
     <row r="103">
-      <c r="A103" t="inlineStr">
+      <c r="A103" s="27" t="inlineStr">
         <is>
           <t>H-02</t>
         </is>
       </c>
-      <c r="B103" t="inlineStr">
+      <c r="B103" s="27" t="inlineStr">
         <is>
           <t>Editorial</t>
         </is>
       </c>
-      <c r="C103" t="inlineStr">
+      <c r="C103" s="27" t="inlineStr">
         <is>
           <t>Pioneros de la publicidad en México</t>
         </is>
       </c>
-      <c r="D103" t="inlineStr">
+      <c r="D103" s="27" t="inlineStr">
         <is>
           <t>Estrategia de marketing y contenidos</t>
         </is>
       </c>
-      <c r="E103" t="inlineStr">
+      <c r="E103" s="27" t="inlineStr">
         <is>
           <t>pioneros de la publicidad en méxico</t>
         </is>
       </c>
-      <c r="F103" t="inlineStr">
+      <c r="F103" s="27" t="inlineStr">
         <is>
           <t>Informacional</t>
         </is>
       </c>
-      <c r="G103" t="inlineStr">
+      <c r="G103" s="27" t="inlineStr">
         <is>
           <t>TOFU</t>
         </is>
       </c>
-      <c r="H103" t="inlineStr">
+      <c r="H103" s="27" t="inlineStr">
         <is>
           <t>Conservar el posicionamiento ya ganado de la URL original (48 clics/16m) con una versión 2026 ampliada y verificada.</t>
         </is>
       </c>
-      <c r="I103" t="inlineStr">
+      <c r="I103" s="27" t="inlineStr">
         <is>
           <t>General</t>
         </is>
       </c>
-      <c r="J103" t="inlineStr">
+      <c r="J103" s="27" t="inlineStr">
         <is>
           <t>México</t>
         </is>
       </c>
-      <c r="K103" t="inlineStr">
+      <c r="K103" s="27" t="inlineStr">
         <is>
           <t>Actualizar v2026 (misma URL)</t>
         </is>
       </c>
-      <c r="L103" t="inlineStr">
+      <c r="L103" s="27" t="inlineStr">
         <is>
           <t>https://www.continentalmedia.com.mx/2014/02/pioneros-de-la-publicidad-en-mexico/</t>
         </is>
       </c>
-      <c r="N103" t="inlineStr">
+      <c r="N103" s="27" t="inlineStr">
         <is>
           <t>Migración SEO — ruta heredada, ver migracion/LEEME_transicion_seo.md §5</t>
         </is>
       </c>
-      <c r="P103" t="inlineStr">
+      <c r="P103" s="27" t="inlineStr">
         <is>
           <t>Estrategia de marketing 360</t>
         </is>
       </c>
-      <c r="R103" t="inlineStr">
+      <c r="R103" s="27" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="T103">
+      <c r="T103" s="27">
         <f>CHOOSE(MONTH(X103),"Ene","Feb","Mar","Abr","May","Jun","Jul","Ago","Sep","Oct","Nov","Dic")&amp;" "&amp;YEAR(X103)</f>
         <v/>
       </c>
-      <c r="W103" t="inlineStr">
-        <is>
-          <t>En revisión</t>
+      <c r="W103" s="27" t="inlineStr">
+        <is>
+          <t>Publicado</t>
         </is>
       </c>
       <c r="X103" s="49" t="n">
         <v>46322</v>
       </c>
-      <c r="Y103">
+      <c r="Y103" s="27">
         <f>CHOOSE(WEEKDAY(X103,2),"lunes","martes","miércoles","jueves","viernes","sábado","domingo")</f>
         <v/>
       </c>
-      <c r="Z103">
+      <c r="Z103" s="27">
         <f>INT((X103-MIN($X$2:$X$103))/7)+1</f>
         <v/>
       </c>
-      <c r="AA103">
+      <c r="AA103" s="27">
         <f>IF(X103=MIN($X$2:$X$103),"Lanzamiento","Calendario semanal")</f>
         <v/>
       </c>
@@ -27106,7 +27106,6 @@
         <v/>
       </c>
     </row>
-    <row r="12"/>
     <row r="13" ht="15" customHeight="1" s="28">
       <c r="A13" s="30" t="inlineStr">
         <is>

</xml_diff>